<commit_message>
Remove Gap Summary sheet from tables.xlsx
https://claude.ai/code/session_012nRaJtG1sRiwbxm8x6EkXT
</commit_message>
<xml_diff>
--- a/data/tables.xlsx
+++ b/data/tables.xlsx
@@ -7,12 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gap Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Simulation - Existing" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Simulation - Proposed" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Block Mapping" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Course Distribution" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Student Analysis" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Simulation - Existing" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Simulation - Proposed" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Block Mapping" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Course Distribution" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Student Analysis" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,17 +428,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Existing (min)</t>
+          <t>Mean (min)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Proposed (min)</t>
+          <t>Median (min)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Delta (min)</t>
+          <t>p25 (min)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>p75 (min)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Max (min)</t>
         </is>
       </c>
     </row>
@@ -450,13 +459,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>346.2</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="D2" t="n">
-        <v>-90</v>
+        <v>290</v>
+      </c>
+      <c r="E2" t="n">
+        <v>400</v>
+      </c>
+      <c r="F2" t="n">
+        <v>660</v>
       </c>
     </row>
     <row r="3">
@@ -466,13 +481,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>260</v>
+        <v>320.1</v>
       </c>
       <c r="C3" t="n">
-        <v>165</v>
+        <v>320</v>
       </c>
       <c r="D3" t="n">
-        <v>-95</v>
+        <v>320</v>
+      </c>
+      <c r="E3" t="n">
+        <v>430</v>
+      </c>
+      <c r="F3" t="n">
+        <v>660</v>
       </c>
     </row>
     <row r="4">
@@ -482,13 +503,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>90</v>
+        <v>346.2</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="D4" t="n">
-        <v>-90</v>
+        <v>290</v>
+      </c>
+      <c r="E4" t="n">
+        <v>400</v>
+      </c>
+      <c r="F4" t="n">
+        <v>660</v>
       </c>
     </row>
     <row r="5">
@@ -498,13 +525,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>319.6</v>
       </c>
       <c r="C5" t="n">
-        <v>165</v>
+        <v>320</v>
       </c>
       <c r="D5" t="n">
-        <v>155</v>
+        <v>320</v>
+      </c>
+      <c r="E5" t="n">
+        <v>430</v>
+      </c>
+      <c r="F5" t="n">
+        <v>430</v>
       </c>
     </row>
     <row r="6">
@@ -514,29 +547,233 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>368.5</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="D6" t="n">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Weekly Total</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+        <v>330</v>
+      </c>
+      <c r="E6" t="n">
+        <v>400</v>
+      </c>
+      <c r="F6" t="n">
         <v>480</v>
       </c>
-      <c r="C7" t="n">
-        <v>330</v>
-      </c>
-      <c r="D7" t="n">
-        <v>-150</v>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Attempts</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Conflicts</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3448</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Conflict rate (%)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Valid schedules</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6552</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mean weekly free (min)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1700.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Median weekly free (min)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1840</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Std dev (min)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>390.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>p25 (min)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>p75 (min)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Min (min)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Max (min)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2510</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Students</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mean (hrs)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Median (hrs)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Min (hrs)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Max (hrs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="n">
+        <v>2707</v>
+      </c>
+      <c r="C22" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="D22" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>16.17</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2246</v>
+      </c>
+      <c r="C23" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="D23" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="E23" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>20.17</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C24" t="n">
+        <v>18.39</v>
+      </c>
+      <c r="D24" t="n">
+        <v>18</v>
+      </c>
+      <c r="E24" t="n">
+        <v>16.17</v>
+      </c>
+      <c r="F24" t="n">
+        <v>25.17</v>
       </c>
     </row>
   </sheetData>
@@ -592,16 +829,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>346.2</v>
+        <v>405.5</v>
       </c>
       <c r="C2" t="n">
-        <v>340</v>
+        <v>420</v>
       </c>
       <c r="D2" t="n">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="E2" t="n">
-        <v>400</v>
+        <v>490</v>
       </c>
       <c r="F2" t="n">
         <v>660</v>
@@ -614,19 +851,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>320.1</v>
+        <v>307.6</v>
       </c>
       <c r="C3" t="n">
-        <v>320</v>
+        <v>390</v>
       </c>
       <c r="D3" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="F3" t="n">
-        <v>660</v>
+        <v>570</v>
       </c>
     </row>
     <row r="4">
@@ -636,16 +873,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>346.2</v>
+        <v>405.1</v>
       </c>
       <c r="C4" t="n">
-        <v>340</v>
+        <v>420</v>
       </c>
       <c r="D4" t="n">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="E4" t="n">
-        <v>400</v>
+        <v>490</v>
       </c>
       <c r="F4" t="n">
         <v>660</v>
@@ -658,19 +895,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>319.6</v>
+        <v>307.6</v>
       </c>
       <c r="C5" t="n">
-        <v>320</v>
+        <v>390</v>
       </c>
       <c r="D5" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="F5" t="n">
-        <v>430</v>
+        <v>570</v>
       </c>
     </row>
     <row r="6">
@@ -680,19 +917,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>368.5</v>
+        <v>405.8</v>
       </c>
       <c r="C6" t="n">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="D6" t="n">
         <v>330</v>
       </c>
       <c r="E6" t="n">
-        <v>400</v>
+        <v>490</v>
       </c>
       <c r="F6" t="n">
-        <v>480</v>
+        <v>660</v>
       </c>
     </row>
     <row r="8">
@@ -724,7 +961,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3448</v>
+        <v>6566</v>
       </c>
     </row>
     <row r="11">
@@ -734,7 +971,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>34.5</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="12">
@@ -744,7 +981,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6552</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="13">
@@ -754,7 +991,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1700.5</v>
+        <v>1831.6</v>
       </c>
     </row>
     <row r="14">
@@ -764,7 +1001,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1840</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="15">
@@ -774,7 +1011,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>390.5</v>
+        <v>544.9</v>
       </c>
     </row>
     <row r="16">
@@ -784,7 +1021,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1620</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="17">
@@ -794,7 +1031,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2030</v>
+        <v>2260</v>
       </c>
     </row>
     <row r="18">
@@ -804,7 +1041,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>300</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19">
@@ -814,7 +1051,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2510</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="21">
@@ -854,19 +1091,19 @@
         <v>3</v>
       </c>
       <c r="B22" t="n">
-        <v>2707</v>
+        <v>1938</v>
       </c>
       <c r="C22" t="n">
-        <v>11.19</v>
+        <v>12.85</v>
       </c>
       <c r="D22" t="n">
-        <v>10.83</v>
+        <v>12.67</v>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="F22" t="n">
-        <v>16.17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23">
@@ -874,19 +1111,19 @@
         <v>4</v>
       </c>
       <c r="B23" t="n">
-        <v>2246</v>
+        <v>1061</v>
       </c>
       <c r="C23" t="n">
-        <v>14.8</v>
+        <v>16.8</v>
       </c>
       <c r="D23" t="n">
-        <v>14.33</v>
+        <v>16.33</v>
       </c>
       <c r="E23" t="n">
-        <v>13.5</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>20.17</v>
+        <v>27.33</v>
       </c>
     </row>
     <row r="24">
@@ -894,19 +1131,19 @@
         <v>5</v>
       </c>
       <c r="B24" t="n">
-        <v>1599</v>
+        <v>435</v>
       </c>
       <c r="C24" t="n">
-        <v>18.39</v>
+        <v>20.36</v>
       </c>
       <c r="D24" t="n">
-        <v>18</v>
+        <v>19.83</v>
       </c>
       <c r="E24" t="n">
-        <v>16.17</v>
+        <v>12.5</v>
       </c>
       <c r="F24" t="n">
-        <v>25.17</v>
+        <v>31.83</v>
       </c>
     </row>
   </sheetData>
@@ -920,363 +1157,515 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Existing Block</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Mean (min)</t>
+          <t>Courses (of 500)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Median (min)</t>
+          <t>→ Proposed Block</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>p25 (min)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>p75 (min)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Max (min)</t>
+          <t>Distance</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>TR long block B</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>405.5</v>
-      </c>
-      <c r="C2" t="n">
-        <v>420</v>
+        <v>64</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TR 100min B</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>330</v>
-      </c>
-      <c r="E2" t="n">
-        <v>490</v>
-      </c>
-      <c r="F2" t="n">
-        <v>660</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>MWF Standard B</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>307.6</v>
-      </c>
-      <c r="C3" t="n">
-        <v>390</v>
+        <v>62</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MWF 50min A</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>465</v>
-      </c>
-      <c r="F3" t="n">
-        <v>570</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>TR long block C</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>405.1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>420</v>
+        <v>60</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TR 75min D</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>330</v>
-      </c>
-      <c r="E4" t="n">
-        <v>490</v>
-      </c>
-      <c r="F4" t="n">
-        <v>660</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>MWF Standard C</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>307.6</v>
-      </c>
-      <c r="C5" t="n">
-        <v>390</v>
+        <v>52</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MWF 50min C</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>465</v>
-      </c>
-      <c r="F5" t="n">
-        <v>570</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>MWF Standard E</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>405.8</v>
-      </c>
-      <c r="C6" t="n">
-        <v>420</v>
+        <v>44</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MWF 70min D</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>330</v>
-      </c>
-      <c r="E6" t="n">
-        <v>490</v>
-      </c>
-      <c r="F6" t="n">
-        <v>660</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MWF Standard F</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>37</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MWF 50min G</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>MW long block A</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>33</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MW 140min B</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Attempts</t>
+          <t>MWF Standard A</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10000</v>
+        <v>28</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MWF 70min A</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Conflicts</t>
+          <t>MWF Standard D</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6566</v>
+        <v>20</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MWF 50min D</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Conflict rate (%)</t>
+          <t>MW long block B</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>65.7</v>
+        <v>19</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MW 140min C</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Valid schedules</t>
+          <t>TR long block A</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3434</v>
+        <v>17</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TR 100min A</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mean weekly free (min)</t>
+          <t>MW Advanced Art Studio A-2</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1831.6</v>
+        <v>9</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MW 170min A</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Median weekly free (min)</t>
+          <t>MWF 3-day long block B</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1950</v>
+        <v>9</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MWF 50min C</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Std dev (min)</t>
+          <t>MWF 3-day long block C</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>544.9</v>
+        <v>7</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MWF 50min G</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>p25 (min)</t>
+          <t>MW Extended Block B</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>6</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MW 170min C</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>p75 (min)</t>
+          <t>MW long block D</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2260</v>
+        <v>5</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MW 140min A</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Min (min)</t>
+          <t>MW long block E</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>160</v>
+        <v>5</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MW 140min A</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Max (min)</t>
+          <t>MWF 3-day long block A</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2970</v>
+        <v>4</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MWF 70min A</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MWF Standard G</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MWF 70min F</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Classes</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Students</t>
-        </is>
+          <t>TR Advanced Art Studio A-3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mean (hrs)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Median (hrs)</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Min (hrs)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Max (hrs)</t>
-        </is>
+          <t>TR 170min A</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MW long block C</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
         <v>3</v>
       </c>
-      <c r="B22" t="n">
-        <v>1938</v>
-      </c>
-      <c r="C22" t="n">
-        <v>12.85</v>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MW 140min D</t>
+        </is>
       </c>
       <c r="D22" t="n">
-        <v>12.67</v>
-      </c>
-      <c r="E22" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F22" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>4</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TR extended block A</t>
+        </is>
       </c>
       <c r="B23" t="n">
-        <v>1061</v>
-      </c>
-      <c r="C23" t="n">
-        <v>16.8</v>
+        <v>3</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TR 170min A</t>
+        </is>
       </c>
       <c r="D23" t="n">
-        <v>16.33</v>
-      </c>
-      <c r="E23" t="n">
         <v>10</v>
       </c>
-      <c r="F23" t="n">
-        <v>27.33</v>
-      </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TR extended block B</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TR 170min B</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MW Extended Block A</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MW 170min A</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TR Experiential Lab Block A-2</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TR 170min A</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TR Experiential Lab Block A-3</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TR 170min A</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
         <v>5</v>
       </c>
-      <c r="B24" t="n">
-        <v>435</v>
-      </c>
-      <c r="C24" t="n">
-        <v>20.36</v>
-      </c>
-      <c r="D24" t="n">
-        <v>19.83</v>
-      </c>
-      <c r="E24" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="F24" t="n">
-        <v>31.83</v>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Tuesday Astronomy Lab</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TR 180min A</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1290,7 +1679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1301,17 +1690,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Courses (of 500)</t>
+          <t>Existing Courses</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>→ Proposed Block</t>
+          <t>Existing %</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Distance</t>
+          <t>Proposed Block</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Proposed Courses</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Proposed %</t>
         </is>
       </c>
     </row>
@@ -1324,13 +1723,19 @@
       <c r="B2" t="n">
         <v>64</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>TR 100min B</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>25</v>
+      <c r="E2" t="n">
+        <v>64</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12.8</v>
       </c>
     </row>
     <row r="3">
@@ -1342,13 +1747,19 @@
       <c r="B3" t="n">
         <v>62</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>MWF 50min A</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>30</v>
+      <c r="E3" t="n">
+        <v>62</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12.4</v>
       </c>
     </row>
     <row r="4">
@@ -1360,13 +1771,19 @@
       <c r="B4" t="n">
         <v>60</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TR 75min D</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>35</v>
+      <c r="C4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MWF 50min C</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>61</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12.2</v>
       </c>
     </row>
     <row r="5">
@@ -1378,13 +1795,19 @@
       <c r="B5" t="n">
         <v>52</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>MWF 50min C</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>10</v>
+      <c r="C5" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TR 75min D</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>60</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -1396,13 +1819,19 @@
       <c r="B6" t="n">
         <v>44</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>MWF 70min D</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>20</v>
+      <c r="E6" t="n">
+        <v>44</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1414,13 +1843,19 @@
       <c r="B7" t="n">
         <v>37</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>MWF 50min G</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>10</v>
+      <c r="E7" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1432,13 +1867,19 @@
       <c r="B8" t="n">
         <v>33</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>MW 140min B</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>25</v>
+      <c r="E8" t="n">
+        <v>33</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.6</v>
       </c>
     </row>
     <row r="9">
@@ -1450,13 +1891,19 @@
       <c r="B9" t="n">
         <v>28</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>MWF 70min A</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>30</v>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.4</v>
       </c>
     </row>
     <row r="10">
@@ -1468,13 +1915,19 @@
       <c r="B10" t="n">
         <v>20</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>MWF 50min D</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>10</v>
+      <c r="E10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1486,13 +1939,19 @@
       <c r="B11" t="n">
         <v>19</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>MW 140min C</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>45</v>
+      <c r="E11" t="n">
+        <v>19</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="12">
@@ -1504,13 +1963,19 @@
       <c r="B12" t="n">
         <v>17</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>TR 100min A</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>25</v>
+      <c r="E12" t="n">
+        <v>17</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="13">
@@ -1522,13 +1987,19 @@
       <c r="B13" t="n">
         <v>9</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>MW 170min A</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
+      <c r="C13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MW 140min A</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1540,13 +2011,19 @@
       <c r="B14" t="n">
         <v>9</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>MWF 50min C</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>40</v>
+      <c r="C14" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MW 170min A</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1558,13 +2035,19 @@
       <c r="B15" t="n">
         <v>7</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MWF 50min G</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>40</v>
+      <c r="C15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TR 170min A</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="16">
@@ -1576,13 +2059,19 @@
       <c r="B16" t="n">
         <v>6</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>MW 170min C</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>20</v>
+      <c r="E16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="17">
@@ -1594,13 +2083,19 @@
       <c r="B17" t="n">
         <v>5</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>MW 140min A</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>75</v>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MWF 70min F</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="18">
@@ -1612,13 +2107,19 @@
       <c r="B18" t="n">
         <v>5</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>MW 140min A</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>35</v>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MW 140min D</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="19">
@@ -1630,13 +2131,19 @@
       <c r="B19" t="n">
         <v>4</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>MWF 70min A</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>40</v>
+      <c r="C19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TR 170min B</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="20">
@@ -1648,12 +2155,18 @@
       <c r="B20" t="n">
         <v>4</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>MWF 70min F</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="C20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TR 180min A</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1666,14 +2179,12 @@
       <c r="B21" t="n">
         <v>4</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>TR 170min A</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>15</v>
-      </c>
+      <c r="C21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1684,14 +2195,12 @@
       <c r="B22" t="n">
         <v>3</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MW 140min D</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>45</v>
-      </c>
+      <c r="C22" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1702,14 +2211,12 @@
       <c r="B23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>TR 170min A</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>10</v>
-      </c>
+      <c r="C23" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1720,14 +2227,12 @@
       <c r="B24" t="n">
         <v>3</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>TR 170min B</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
+      <c r="C24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1738,14 +2243,12 @@
       <c r="B25" t="n">
         <v>1</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MW 170min A</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>25</v>
-      </c>
+      <c r="C25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1756,14 +2259,12 @@
       <c r="B26" t="n">
         <v>1</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>TR 170min A</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>25</v>
-      </c>
+      <c r="C26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1774,14 +2275,12 @@
       <c r="B27" t="n">
         <v>0</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>TR 170min A</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>5</v>
-      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1792,14 +2291,12 @@
       <c r="B28" t="n">
         <v>0</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>TR 180min A</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>110</v>
-      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1812,636 +2309,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Existing Block</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Existing Courses</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Existing %</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Proposed Block</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Proposed Courses</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Proposed %</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TR long block B</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>64</v>
-      </c>
-      <c r="C2" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TR 100min B</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>64</v>
-      </c>
-      <c r="F2" t="n">
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MWF Standard B</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>62</v>
-      </c>
-      <c r="C3" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>MWF 50min A</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>62</v>
-      </c>
-      <c r="F3" t="n">
-        <v>12.4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TR long block C</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>60</v>
-      </c>
-      <c r="C4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>MWF 50min C</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>61</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MWF Standard C</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>52</v>
-      </c>
-      <c r="C5" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>TR 75min D</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>60</v>
-      </c>
-      <c r="F5" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MWF Standard E</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>44</v>
-      </c>
-      <c r="C6" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>MWF 70min D</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>44</v>
-      </c>
-      <c r="F6" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MWF Standard F</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>37</v>
-      </c>
-      <c r="C7" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>MWF 50min G</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>44</v>
-      </c>
-      <c r="F7" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>MW long block A</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>33</v>
-      </c>
-      <c r="C8" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>MW 140min B</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>33</v>
-      </c>
-      <c r="F8" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>MWF Standard A</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>28</v>
-      </c>
-      <c r="C9" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MWF 70min A</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>32</v>
-      </c>
-      <c r="F9" t="n">
-        <v>6.4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MWF Standard D</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>MWF 50min D</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>MW long block B</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>19</v>
-      </c>
-      <c r="C11" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>MW 140min C</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>19</v>
-      </c>
-      <c r="F11" t="n">
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TR long block A</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>17</v>
-      </c>
-      <c r="C12" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>TR 100min A</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>17</v>
-      </c>
-      <c r="F12" t="n">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MW Advanced Art Studio A-2</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>9</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>MW 140min A</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MWF 3-day long block B</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>9</v>
-      </c>
-      <c r="C14" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>MW 170min A</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>10</v>
-      </c>
-      <c r="F14" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>MWF 3-day long block C</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>7</v>
-      </c>
-      <c r="C15" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>TR 170min A</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>8</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>MW Extended Block B</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>6</v>
-      </c>
-      <c r="C16" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MW 170min C</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>MW long block D</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MWF 70min F</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>MW long block E</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MW 140min D</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>MWF 3-day long block A</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>4</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>TR 170min B</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>MWF Standard G</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>TR 180min A</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TR Advanced Art Studio A-3</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>4</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>MW long block C</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TR extended block A</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>3</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TR extended block B</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>3</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>MW Extended Block A</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>TR Experiential Lab Block A-2</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>TR Experiential Lab Block A-3</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Tuesday Astronomy Lab</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>